<commit_message>
Change term model.dll and logic.dll become XenAnalyticDevice.dll and XenAnalyticModel.dll
</commit_message>
<xml_diff>
--- a/Training_model/supplementary/XenIdentifier Project Timeline.xlsx
+++ b/Training_model/supplementary/XenIdentifier Project Timeline.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DeviceIdentifier\1.Training_model\supplementary\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DeviceIdentifier\Training_model\supplementary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44094F06-DF23-42EE-9591-A51DBAB88183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C48D403-E6FE-4636-9175-3CFD49363E12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="81">
   <si>
     <t>Date</t>
   </si>
@@ -264,13 +264,61 @@
     <t>EQUIPMENT TYPE = Logic function – no model involved; 
 Script “predict_equipment.py”; Integrated inside C#; 
 Section and Cluster = XGBoost Model; Proceed as previous model</t>
+  </si>
+  <si>
+    <t>September</t>
+  </si>
+  <si>
+    <r>
+      <t>Refine</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Reference\DeviceIdentifier-API-FullReference.docx"</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Align with format given by Stanley at this file :</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "C:\Users\sitisyaziyah\Downloads\General » xenDBLink v1 2.docx"</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Rename dll library : 
+Logic.dll -&gt; XenAnalyticDevice.dll 
+Model.dll -&gt; XenAnalyticModel.dll 
+Service.py -&gt; XenAnalyticService.py </t>
+  </si>
+  <si>
+    <t># change the readme markdown file?
+# DeviceIdentifier-API-FullReference.docx</t>
+  </si>
+  <si>
+    <t>Update MSTeams Planner</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -295,6 +343,14 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="12">
@@ -376,17 +432,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -422,6 +472,27 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -809,605 +880,653 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.26953125" customWidth="1"/>
-    <col min="2" max="2" width="16" style="6" customWidth="1"/>
-    <col min="3" max="3" width="42" customWidth="1"/>
-    <col min="4" max="4" width="69.36328125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="17.26953125" style="4" customWidth="1"/>
+    <col min="2" max="2" width="16" style="4" customWidth="1"/>
+    <col min="3" max="3" width="54" customWidth="1"/>
+    <col min="4" max="4" width="69.36328125" style="2" customWidth="1"/>
     <col min="5" max="5" width="22.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="16" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="3" t="str">
         <f>TEXT(A2,"mmmm")</f>
         <v>July</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="5" t="str">
+      <c r="B3" s="3" t="str">
         <f t="shared" ref="B3:B34" si="0">TEXT(A3,"mmmm")</f>
         <v>July</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="6" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="5" t="str">
+      <c r="B4" s="3" t="str">
         <f t="shared" si="0"/>
         <v>July</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="E4" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="B5" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="58" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="E5" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="B6" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="6" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="B7" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="9" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="B8" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="8" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="B9" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="E9" s="12" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+      <c r="E9" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="B10" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="10" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="B11" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="10" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="B12" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C13" s="2" t="s">
+      <c r="B13" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="13" t="s">
+      <c r="D13" s="1"/>
+      <c r="E13" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="B14" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="13" t="s">
+      <c r="D14" s="1"/>
+      <c r="E14" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="B15" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="13" t="s">
+      <c r="E15" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C16" s="2" t="s">
+      <c r="B16" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="13" t="s">
+      <c r="E16" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C17" s="2" t="s">
+      <c r="B17" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="2"/>
-      <c r="E17" s="13" t="s">
+      <c r="D17" s="1"/>
+      <c r="E17" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C18" s="2" t="s">
+      <c r="B18" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D18" s="2"/>
-      <c r="E18" s="13" t="s">
+      <c r="D18" s="1"/>
+      <c r="E18" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C19" s="2" t="s">
+      <c r="B19" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A20" s="2" t="s">
+      <c r="D19" s="1"/>
+      <c r="E19" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C20" s="2" t="s">
+      <c r="B20" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="2"/>
-      <c r="E20" s="13" t="s">
+      <c r="D20" s="1"/>
+      <c r="E20" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C21" s="2" t="s">
+      <c r="B21" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D21" s="2"/>
-      <c r="E21" s="13" t="s">
+      <c r="D21" s="1"/>
+      <c r="E21" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C22" s="2" t="s">
+      <c r="B22" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B23" s="5" t="str">
+      <c r="B23" s="3" t="str">
         <f t="shared" si="0"/>
         <v>PENDING</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D23" s="2"/>
-      <c r="E23" s="15" t="s">
+      <c r="D23" s="1"/>
+      <c r="E23" s="13" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B24" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C24" s="2" t="s">
+      <c r="B24" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D24" s="2"/>
-      <c r="E24" s="13" t="s">
+      <c r="D24" s="1"/>
+      <c r="E24" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B25" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C25" s="2" t="s">
+      <c r="B25" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D25" s="2"/>
-      <c r="E25" s="13" t="s">
+      <c r="D25" s="1"/>
+      <c r="E25" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="87" x14ac:dyDescent="0.35">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B26" s="5" t="str">
+      <c r="B26" s="3" t="str">
         <f t="shared" si="0"/>
         <v>September</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D26" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="E26" s="13" t="s">
+      <c r="E26" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A27" s="2" t="s">
+      <c r="A27" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B27" s="5" t="str">
+      <c r="B27" s="3" t="str">
         <f t="shared" si="0"/>
         <v>September</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D27" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E27" s="13" t="s">
+      <c r="E27" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B28" s="5" t="str">
+      <c r="B28" s="3" t="str">
         <f t="shared" si="0"/>
         <v>September</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D28" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E28" s="13" t="s">
+      <c r="E28" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="58" x14ac:dyDescent="0.35">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B29" s="5" t="str">
+      <c r="B29" s="3" t="str">
         <f t="shared" si="0"/>
         <v>September</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="D29" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E29" s="13" t="s">
+      <c r="E29" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B30" s="5" t="str">
+      <c r="B30" s="3" t="str">
         <f t="shared" si="0"/>
         <v>September</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="D30" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E30" s="13" t="s">
+      <c r="E30" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="5" t="str">
+      <c r="B31" s="3" t="str">
         <f t="shared" si="0"/>
         <v>September</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D31" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E31" s="13" t="s">
+      <c r="E31" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B32" s="5" t="str">
+      <c r="B32" s="3" t="str">
         <f t="shared" si="0"/>
         <v>September</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D32" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E32" s="13" t="s">
+      <c r="E32" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B33" s="5" t="str">
+      <c r="B33" s="3" t="str">
         <f t="shared" si="0"/>
         <v>September</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="D33" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E33" s="13" t="s">
+      <c r="E33" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34" s="2" t="s">
+      <c r="A34" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B34" s="5" t="str">
+      <c r="B34" s="3" t="str">
         <f t="shared" si="0"/>
         <v>September</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C34" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="D34" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="E34" s="14" t="s">
-        <v>25</v>
+      <c r="E34" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A35" s="18">
+        <v>46286</v>
+      </c>
+      <c r="B35" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A36" s="18">
+        <v>46286</v>
+      </c>
+      <c r="B36" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="E36" s="15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37" s="20">
+        <v>46287</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C37" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="E37" s="15" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rename Model.dll and Logic.dll
</commit_message>
<xml_diff>
--- a/Training_model/supplementary/XenIdentifier Project Timeline.xlsx
+++ b/Training_model/supplementary/XenIdentifier Project Timeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DeviceIdentifier\Training_model\supplementary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C48D403-E6FE-4636-9175-3CFD49363E12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD549B5-CF8A-468E-BD16-0649D23F0073}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Progress" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
convert compatibe mode into docs
</commit_message>
<xml_diff>
--- a/Training_model/supplementary/XenIdentifier Project Timeline.xlsx
+++ b/Training_model/supplementary/XenIdentifier Project Timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DeviceIdentifier\Training_model\supplementary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD549B5-CF8A-468E-BD16-0649D23F0073}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21DEE7D8-A4C4-4604-8D4A-A13F2FEF563D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,9 +57,6 @@
     <t>Stage 1 - Stage 3</t>
   </si>
   <si>
-    <t>Pending on Stanley review</t>
-  </si>
-  <si>
     <t>Refer to the slide “Movement of dataset [UPDATE 04/08/26]”</t>
   </si>
   <si>
@@ -313,12 +310,15 @@
   <si>
     <t>Update MSTeams Planner</t>
   </si>
+  <si>
+    <t>Pending Work</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -330,12 +330,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -353,7 +347,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -372,42 +366,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA9D18E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9E1F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFE699"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8CBAD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF9DC3E6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFBDD7EE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF4CCCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -432,7 +392,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -446,38 +406,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -494,19 +427,17 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D9D9"/>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -520,14 +451,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FF9BFFBC"/>
           <bgColor rgb="FF99FFCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9DC3E6"/>
-          <bgColor theme="6" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -886,24 +809,24 @@
     <col min="1" max="1" width="17.26953125" style="4" customWidth="1"/>
     <col min="2" max="2" width="16" style="4" customWidth="1"/>
     <col min="3" max="3" width="54" customWidth="1"/>
-    <col min="4" max="4" width="69.36328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="55.453125" style="2" customWidth="1"/>
     <col min="5" max="5" width="22.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="C1" s="16" t="s">
+      <c r="B1" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" s="7" t="s">
         <v>3</v>
       </c>
     </row>
@@ -916,13 +839,13 @@
         <v>July</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -934,13 +857,13 @@
         <v>July</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>25</v>
+        <v>6</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -952,620 +875,617 @@
         <v>July</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>25</v>
+        <v>7</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>25</v>
+      <c r="E5" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" s="3" t="str">
         <f t="shared" si="0"/>
         <v>August</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>25</v>
+        <v>10</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>25</v>
+      <c r="E7" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8" s="3" t="str">
         <f t="shared" si="0"/>
         <v>August</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="B9" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E8" s="8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>25</v>
+      <c r="E9" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>25</v>
+      <c r="E10" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="D11" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>25</v>
+        <v>20</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C12" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="D13" s="1"/>
-      <c r="E13" s="11" t="s">
-        <v>25</v>
+      <c r="E13" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14" s="3" t="str">
         <f t="shared" si="0"/>
         <v>August</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D14" s="1"/>
-      <c r="E14" s="11" t="s">
-        <v>25</v>
+      <c r="E14" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B15" s="3" t="str">
         <f t="shared" si="0"/>
         <v>August</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="E15" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C16" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A17" s="3" t="s">
+      <c r="B17" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="D17" s="1"/>
-      <c r="E17" s="11" t="s">
-        <v>25</v>
+      <c r="E17" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18" s="3" t="str">
         <f t="shared" si="0"/>
         <v>August</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D18" s="1"/>
-      <c r="E18" s="11" t="s">
-        <v>25</v>
+      <c r="E18" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B19" s="3" t="str">
         <f t="shared" si="0"/>
         <v>August</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D19" s="1"/>
-      <c r="E19" s="11" t="s">
-        <v>25</v>
+      <c r="E19" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B20" s="3" t="str">
         <f t="shared" si="0"/>
         <v>August</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D20" s="1"/>
-      <c r="E20" s="11" t="s">
-        <v>25</v>
+      <c r="E20" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B21" s="3" t="str">
         <f t="shared" si="0"/>
         <v>August</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D21" s="1"/>
-      <c r="E21" s="11" t="s">
-        <v>25</v>
+      <c r="E21" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B22" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C22" s="1" t="s">
+      <c r="D22" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="E22" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="E22" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23" s="3" t="s">
+      <c r="B23" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>PENDING</v>
+      </c>
+      <c r="C23" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="B23" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PENDING</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D23" s="1"/>
-      <c r="E23" s="13" t="s">
-        <v>41</v>
+      <c r="D23" s="13"/>
+      <c r="E23" s="5" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B24" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="D24" s="1"/>
-      <c r="E24" s="11" t="s">
-        <v>25</v>
+      <c r="E24" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B25" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>August</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B25" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>August</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="D25" s="1"/>
-      <c r="E25" s="11" t="s">
-        <v>25</v>
+      <c r="E25" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="87" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>September</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B26" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>September</v>
-      </c>
-      <c r="C26" s="1" t="s">
+      <c r="D26" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D26" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E26" s="11" t="s">
-        <v>25</v>
+      <c r="E26" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B27" s="3" t="str">
         <f t="shared" si="0"/>
         <v>September</v>
       </c>
       <c r="C27" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D27" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E27" s="11" t="s">
-        <v>25</v>
+      <c r="E27" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B28" s="3" t="str">
         <f t="shared" si="0"/>
         <v>September</v>
       </c>
       <c r="C28" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="E28" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A29" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B29" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>September</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E28" s="11" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="58" x14ac:dyDescent="0.35">
-      <c r="A29" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B29" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>September</v>
-      </c>
-      <c r="C29" s="1" t="s">
+      <c r="D29" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D29" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="E29" s="11" t="s">
-        <v>25</v>
+      <c r="E29" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>September</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B30" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>September</v>
-      </c>
-      <c r="C30" s="1" t="s">
+      <c r="D30" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D30" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="E30" s="11" t="s">
-        <v>25</v>
+      <c r="E30" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B31" s="3" t="str">
         <f t="shared" si="0"/>
         <v>September</v>
       </c>
       <c r="C31" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D31" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="E31" s="11" t="s">
-        <v>25</v>
+      <c r="E31" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B32" s="3" t="str">
         <f t="shared" si="0"/>
         <v>September</v>
       </c>
       <c r="C32" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D32" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>25</v>
+      <c r="E32" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B33" s="3" t="str">
         <f t="shared" si="0"/>
         <v>September</v>
       </c>
       <c r="C33" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D33" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D33" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E33" s="11" t="s">
-        <v>25</v>
+      <c r="E33" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>September</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B34" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>September</v>
-      </c>
-      <c r="C34" s="1" t="s">
+      <c r="D34" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D34" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E34" s="12" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A35" s="18">
+      <c r="E34" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A35" s="9">
         <v>46286</v>
       </c>
-      <c r="B35" s="19" t="s">
+      <c r="B35" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="C35" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C35" s="14" t="s">
+      <c r="D35" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="D35" s="14" t="s">
+      <c r="E35" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A36" s="9">
+        <v>46286</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E35" s="15" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="58" x14ac:dyDescent="0.35">
-      <c r="A36" s="18">
-        <v>46286</v>
-      </c>
-      <c r="B36" s="19" t="s">
-        <v>75</v>
-      </c>
-      <c r="C36" s="2" t="s">
+      <c r="D36" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D36" s="14" t="s">
+      <c r="E36" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37" s="11">
+        <v>46287</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C37" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="E36" s="15" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37" s="20">
-        <v>46287</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C37" s="14" t="s">
+      <c r="E37" s="5" t="s">
         <v>80</v>
-      </c>
-      <c r="E37" s="15" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E34" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="E2:E999">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
-      <formula>"Pending on Stanley review"</formula>
+    <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
+      <formula>"Pending Review"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
       <formula>"Completed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
-      <formula>"On drafting – preparation for training"</formula>
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
+      <formula>"Drafting"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
-      <formula>"In progressing"</formula>
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+      <formula>"In Progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
-      <formula>"In planning; Not execute in coding"</formula>
+    <cfRule type="cellIs" dxfId="2" priority="5" operator="equal">
+      <formula>"Planning"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="6" operator="equal">
-      <formula>"Complete in pipeline C#"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="7" operator="equal">
       <formula>"Synch in Git"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="8" operator="equal">
-      <formula>"PENDING"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="9" operator="equal">
-      <formula>"Current update"</formula>
+    <cfRule type="cellIs" dxfId="0" priority="8" operator="equal">
+      <formula>"Pending Work"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" error="Please select a status from the dropdown list." sqref="E39:E999" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>StatusOptions</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" error="Please select a status from the dropdown list." sqref="E2:E38" xr:uid="{8EA7E1BD-2BD4-4FEA-AC5C-45E553151505}">
-      <formula1>"Pending on Stanley review,Completed,On drafting – preparation for training,In progressing,In planning; Not execute in coding,Complete in pipeline C#,Synch in Git,PENDING,Current update"</formula1>
+    <dataValidation type="list" allowBlank="1" error="Please select a status from the dropdown list." sqref="E38" xr:uid="{8EA7E1BD-2BD4-4FEA-AC5C-45E553151505}">
+      <formula1>"Pending on Stanley review,Completed,On drafting,In progressing,In planning; Not execute in coding,Complete in pipeline C#,Synch in Git,PENDING,Current update"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E37" xr:uid="{169CDA58-BA09-4855-AEDC-9D570CAD6163}">
+      <formula1>"Planning, Drafting, In progress, Completed, Synch in Git, Pending Work, Pending Review"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>